<commit_message>
Session dates, PESTEL criteria search as proposal step with mandatory sources, industry source list template, numbers presented in slides
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkWScMhuRmEB4zppSmB7Ri
</commit_message>
<xml_diff>
--- a/WT26-27/PESTEL Indicator Search Template.xlsx
+++ b/WT26-27/PESTEL Indicator Search Template.xlsx
@@ -615,7 +615,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="70" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -623,7 +623,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Collect indicators that could describe the six countries for a premium coffee launch by Julius Meinl. Search for indicators for each PESTEL dimension first (political, economic, social, technological, environmental, legal). In the next step you shortlist 8 to 14 of them for your scoring model.</t>
+          <t>Step 1 of the scoring method. Search for criteria (indicators) for each PESTEL dimension (political, economic, social, technological, environmental, legal) that could describe the six countries for a premium coffee launch by Julius Meinl. The instructor merges the proposals of all groups and selects the final criteria (5 political, 10 economic, 10 social, 10 technological, 5 environmental, 5 legal). After that, every group enters the raw data of its own country in the shared sheet "Country scoring model". The source is therefore essential: if your criterion is selected, the other groups must be able to find the data for their countries.</t>
         </is>
       </c>
     </row>
@@ -656,28 +656,35 @@
     <row r="9" ht="44" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>4. For every indicator, fill in the definition, source, link and direction. Open the source and check whether data exist for each of the six countries. Set each country to Yes, Partly, No or Not checked. The instructor has not checked coverage: this is your first task.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+          <t>4. For every indicator, fill in the definition, unit, direction, source name and source link. The link opens the page where the data can be downloaded. Open the source and check whether data exist for each of the six countries. Set each country to Yes, Partly, No or Not checked. The instructor has not checked coverage: this is your first task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>5. Rate each indicator for relevance and data quality (1 to 5).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="44" customHeight="1">
+          <t>5. In the column "How to find the data (steps) and comment" write the steps another group needs to find the numbers (for example: open the database, choose the indicator, select the country and the latest year). Qualitative criteria need a rubric with the meaning of the scores 1 to 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>6. Mark 8 to 14 indicators as Shortlist = Yes. Use the Summary tab to check that every dimension and all six Julius Meinl dimensions are represented and that the shortlisted indicators cover all six countries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+          <t>6. Rate each indicator for relevance and data quality (1 to 5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>7. Copy the shortlist into the Criteria sheet of your Excel model.</t>
+          <t>7. Mark your best indicators as Proposal = Yes (the Summary tab shows how many you need). Use the Summary tab to check that every dimension is covered, that every proposal has a source and a link, and that the data exist for all six countries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>8. Submit your sheet by the deadline. The instructor merges all group sheets, selects the final criteria and publishes the sheet "Country scoring model" with the selected criteria. You then enter the numbers of your country there.</t>
         </is>
       </c>
     </row>
@@ -689,7 +696,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>The source link opens the page where the data can be downloaded, not the home page of the publisher.</t>
+          <t>A source name and a working link are required for every proposal. The link opens the page where the data can be downloaded, not the home page of the publisher.</t>
         </is>
       </c>
     </row>
@@ -703,7 +710,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Do not delete the instructor's rows. If you do not use an indicator, leave Shortlist empty and say why in the comment.</t>
+          <t>Do not delete the instructor's rows. If you do not propose an indicator, leave Proposal empty and say why in the comment.</t>
         </is>
       </c>
     </row>
@@ -750,7 +757,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Deadline for the long list</t>
+          <t>Deadline for the proposals</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -925,7 +932,7 @@
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Shortlist?</t>
+          <t>Proposal?</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
@@ -961,12 +968,12 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>How to find the data (steps) and comment</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Use PPP rather than current US dollars to compare spending power.</t>
+          <t>Open WDI, search "GDP per capita, PPP", select the six countries and the latest year. Use PPP rather than current US dollars to compare spending power.</t>
         </is>
       </c>
     </row>
@@ -1325,12 +1332,12 @@
       </c>
       <c r="U1" s="9" t="inlineStr">
         <is>
-          <t>Shortlist?</t>
+          <t>Proposal?</t>
         </is>
       </c>
       <c r="V1" s="9" t="inlineStr">
         <is>
-          <t>Shortlist check</t>
+          <t>Proposal check</t>
         </is>
       </c>
       <c r="W1" s="9" t="inlineStr">
@@ -1350,7 +1357,7 @@
       </c>
       <c r="Z1" s="9" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>How to find the data (steps) and comment</t>
         </is>
       </c>
     </row>
@@ -7440,21 +7447,21 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Shortlist: minimum number of indicators</t>
+          <t>Proposals: minimum number of indicators</t>
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Shortlist: maximum number of indicators</t>
+          <t>Proposals: maximum number of indicators</t>
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
@@ -7475,7 +7482,7 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Shortlisted</t>
+          <t>Proposed</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -7503,7 +7510,7 @@
         <v/>
       </c>
       <c r="E9" s="14">
-        <f>IF(B9&lt;$B$4,"Search for more indicators",IF(D9=0,"Shortlist at least one","OK"))</f>
+        <f>IF(B9&lt;$B$4,"Search for more indicators",IF(D9=0,"Propose at least one","OK"))</f>
         <v/>
       </c>
     </row>
@@ -7526,7 +7533,7 @@
         <v/>
       </c>
       <c r="E10" s="14">
-        <f>IF(B10&lt;$B$4,"Search for more indicators",IF(D10=0,"Shortlist at least one","OK"))</f>
+        <f>IF(B10&lt;$B$4,"Search for more indicators",IF(D10=0,"Propose at least one","OK"))</f>
         <v/>
       </c>
     </row>
@@ -7549,7 +7556,7 @@
         <v/>
       </c>
       <c r="E11" s="14">
-        <f>IF(B11&lt;$B$4,"Search for more indicators",IF(D11=0,"Shortlist at least one","OK"))</f>
+        <f>IF(B11&lt;$B$4,"Search for more indicators",IF(D11=0,"Propose at least one","OK"))</f>
         <v/>
       </c>
     </row>
@@ -7572,7 +7579,7 @@
         <v/>
       </c>
       <c r="E12" s="14">
-        <f>IF(B12&lt;$B$4,"Search for more indicators",IF(D12=0,"Shortlist at least one","OK"))</f>
+        <f>IF(B12&lt;$B$4,"Search for more indicators",IF(D12=0,"Propose at least one","OK"))</f>
         <v/>
       </c>
     </row>
@@ -7595,7 +7602,7 @@
         <v/>
       </c>
       <c r="E13" s="14">
-        <f>IF(B13&lt;$B$4,"Search for more indicators",IF(D13=0,"Shortlist at least one","OK"))</f>
+        <f>IF(B13&lt;$B$4,"Search for more indicators",IF(D13=0,"Propose at least one","OK"))</f>
         <v/>
       </c>
     </row>
@@ -7618,7 +7625,7 @@
         <v/>
       </c>
       <c r="E14" s="14">
-        <f>IF(B14&lt;$B$4,"Search for more indicators",IF(D14=0,"Shortlist at least one","OK"))</f>
+        <f>IF(B14&lt;$B$4,"Search for more indicators",IF(D14=0,"Propose at least one","OK"))</f>
         <v/>
       </c>
     </row>
@@ -7645,11 +7652,11 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Shortlist size</t>
+          <t>Number of proposals</t>
         </is>
       </c>
       <c r="B17" s="14">
-        <f>IF(D15&lt;$B$5,"Too few: shortlist more",IF(D15&gt;$B$6,"Too many: cut down","Within the range"))</f>
+        <f>IF(D15&lt;$B$5,"Too few: propose more",IF(D15&gt;$B$6,"Too many: cut down","Within the range"))</f>
         <v/>
       </c>
       <c r="C17" s="17" t="n"/>
@@ -7657,7 +7664,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Shortlisted indicators without data for all six countries</t>
+          <t>Proposals without data for all six countries</t>
         </is>
       </c>
       <c r="B18" s="14">
@@ -7665,6 +7672,17 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Proposals without source name or link</t>
+        </is>
+      </c>
+      <c r="B19" s="14">
+        <f>COUNTIFS('Long list'!$U$2:$U$100,"Yes",'Long list'!$J$2:$J$100,"")+COUNTIFS('Long list'!$U$2:$U$100,"Yes",'Long list'!$I$2:$I$100,"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
@@ -7673,7 +7691,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Shortlisted indicators</t>
+          <t>Proposed indicators</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Each group finds 45 criteria by session 3; PESTEL sheet targets per dimension
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkWScMhuRmEB4zppSmB7Ri
</commit_message>
<xml_diff>
--- a/WT26-27/PESTEL Indicator Search Template.xlsx
+++ b/WT26-27/PESTEL Indicator Search Template.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Step 1 of the scoring method. Search for criteria (indicators) for each PESTEL dimension (political, economic, social, technological, environmental, legal) that could describe the six countries for a premium coffee launch by Julius Meinl. The instructor merges the proposals of all groups and selects the final criteria (5 political, 10 economic, 10 social, 10 technological, 5 environmental, 5 legal). After that, every group enters the raw data of its own country in the shared sheet "Country scoring model". The source is therefore essential: if your criterion is selected, the other groups must be able to find the data for their countries.</t>
+          <t>Step 1 of the scoring method. Each group finds 45 criteria. Search for criteria (indicators) for each PESTEL dimension (political, economic, social, technological, environmental, legal) that could describe the six countries for a premium coffee launch by Julius Meinl. The instructor merges the proposals of all groups and selects the final criteria (5 political, 10 economic, 10 social, 10 technological, 5 environmental, 5 legal). After that, every group enters the raw data of its own country in the shared sheet "Country scoring model". The source is therefore essential: if your criterion is selected, the other groups must be able to find the data for their countries.</t>
         </is>
       </c>
     </row>
@@ -677,14 +677,14 @@
     <row r="12" ht="44" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>7. Mark your best indicators as Proposal = Yes (the Summary tab shows how many you need). Use the Summary tab to check that every dimension is covered, that every proposal has a source and a link, and that the data exist for all six countries.</t>
+          <t>7. Mark every indicator you propose as Proposal = Yes. You need 45 proposals: 5 political, 10 economic, 10 social, 10 technological, 5 environmental and 5 legal (the Summary tab shows what is still missing). Use the Summary tab to check that every dimension is covered, that every proposal has a source and a link, and that the data exist for all six countries.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>8. Submit your sheet by the deadline. The instructor merges all group sheets, selects the final criteria and publishes the sheet "Country scoring model" with the selected criteria. You then enter the numbers of your country there.</t>
+          <t>8. Submit your sheet by session 3 (Monday 19 October 2026). The instructor merges all group sheets, preselects the final criteria and publishes the sheet "Country scoring model" with the selected criteria. You then enter the numbers of your country there.</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>[date, to be confirmed]</t>
+          <t>Session 3: Monday 19 October 2026</t>
         </is>
       </c>
     </row>
@@ -7409,7 +7409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7437,21 +7437,23 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Minimum candidate indicators per PESTEL dimension</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="n">
-        <v>3</v>
+          <t>Target: indicators to find per dimension</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>See column F (45 in total)</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Proposals: minimum number of indicators</t>
+          <t>Proposals: minimum number of indicators (each group)</t>
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -7461,7 +7463,7 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -7490,6 +7492,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -7510,8 +7517,11 @@
         <v/>
       </c>
       <c r="E9" s="14">
-        <f>IF(B9&lt;$B$4,"Search for more indicators",IF(D9=0,"Propose at least one","OK"))</f>
-        <v/>
+        <f>IF(D9&lt;F9,"Propose "&amp;(F9-D9)&amp;" more","OK")</f>
+        <v/>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -7533,8 +7543,11 @@
         <v/>
       </c>
       <c r="E10" s="14">
-        <f>IF(B10&lt;$B$4,"Search for more indicators",IF(D10=0,"Propose at least one","OK"))</f>
-        <v/>
+        <f>IF(D10&lt;F10,"Propose "&amp;(F10-D10)&amp;" more","OK")</f>
+        <v/>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -7556,8 +7569,11 @@
         <v/>
       </c>
       <c r="E11" s="14">
-        <f>IF(B11&lt;$B$4,"Search for more indicators",IF(D11=0,"Propose at least one","OK"))</f>
-        <v/>
+        <f>IF(D11&lt;F11,"Propose "&amp;(F11-D11)&amp;" more","OK")</f>
+        <v/>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -7579,8 +7595,11 @@
         <v/>
       </c>
       <c r="E12" s="14">
-        <f>IF(B12&lt;$B$4,"Search for more indicators",IF(D12=0,"Propose at least one","OK"))</f>
-        <v/>
+        <f>IF(D12&lt;F12,"Propose "&amp;(F12-D12)&amp;" more","OK")</f>
+        <v/>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -7602,8 +7621,11 @@
         <v/>
       </c>
       <c r="E13" s="14">
-        <f>IF(B13&lt;$B$4,"Search for more indicators",IF(D13=0,"Propose at least one","OK"))</f>
-        <v/>
+        <f>IF(D13&lt;F13,"Propose "&amp;(F13-D13)&amp;" more","OK")</f>
+        <v/>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -7625,8 +7647,11 @@
         <v/>
       </c>
       <c r="E14" s="14">
-        <f>IF(B14&lt;$B$4,"Search for more indicators",IF(D14=0,"Propose at least one","OK"))</f>
-        <v/>
+        <f>IF(D14&lt;F14,"Propose "&amp;(F14-D14)&amp;" more","OK")</f>
+        <v/>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -7648,6 +7673,10 @@
         <v/>
       </c>
       <c r="E15" s="14" t="inlineStr"/>
+      <c r="F15" s="16">
+        <f>SUM(F9:F14)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">

</xml_diff>